<commit_message>
Add DOI links; no data changes (#2)
* Update README.md

* Add link
</commit_message>
<xml_diff>
--- a/data/connector-crosswalk_current.xlsx
+++ b/data/connector-crosswalk_current.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECA37308-F5D2-41C5-B93C-6B1826046830}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A3D29E7-831D-49E2-A4CA-34F0EC736BB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31800" yWindow="3000" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32340" yWindow="2430" windowWidth="21600" windowHeight="11985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data_dictionary" sheetId="3" r:id="rId1"/>
@@ -21332,7 +21332,7 @@
     <t>Attributes about the geography’s associated entity; see above for details</t>
   </si>
   <si>
-    <t xml:space="preserve">  *Users are encouraged to refer to Department of Interior geography–entity crosswalk data products for further detail</t>
+    <t xml:space="preserve">  *Users are encouraged to refer to Department of Interior geography–entity crosswalk data products for further detail: https://github.com/doi-do/census-tribal</t>
   </si>
 </sst>
 </file>

</xml_diff>